<commit_message>
Refactor code structure and optimize performance across multiple modules
</commit_message>
<xml_diff>
--- a/etudecas/data/source/268967.xlsx
+++ b/etudecas/data/source/268967.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://scalian-my.sharepoint.com/personal/yannick_martz_scalian_com/Documents/0_FILES_YM/2026/Pierre Fabre/Data/safe/IN/PF/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{F1B106E4-76CD-4A29-A43F-305A6627139B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D7261265-CC28-47B7-ABF1-966417990AA3}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{F1B106E4-76CD-4A29-A43F-305A6627139B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6281DBA4-2371-4798-8153-31371BEB4561}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM" sheetId="1" r:id="rId1"/>
@@ -220,7 +220,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -246,6 +246,9 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -582,10 +585,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F26"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="22" bestFit="1" customWidth="1"/>
@@ -772,6 +775,9 @@
       <c r="F9" t="s">
         <v>10</v>
       </c>
+    </row>
+    <row r="26" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C26" s="9"/>
     </row>
   </sheetData>
   <autoFilter ref="C1:F9" xr:uid="{00000000-0001-0000-0000-000000000000}">
@@ -790,9 +796,9 @@
   <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="25.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.6640625" customWidth="1"/>
+    <col min="7" max="7" width="11.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -1035,12 +1041,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -1049,9 +1049,9 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002D5C0BAE13F791428A2467AD4E2CA4A9" ma:contentTypeVersion="3" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="e041f94258a4985e0980ebef8737f2c5">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="911fa86e-1244-486f-9d05-850c48c46759" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="44562186199d162c4fe6c5d19537b3b1" ns2:_="">
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002D5C0BAE13F791428A2467AD4E2CA4A9" ma:contentTypeVersion="8" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="2ef8d77b566c9fd80e9c2bdc9338d629">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="911fa86e-1244-486f-9d05-850c48c46759" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="803aa259af1a7fc7d7bef2888f2078ba" ns2:_="">
     <xsd:import namespace="911fa86e-1244-486f-9d05-850c48c46759"/>
     <xsd:element name="properties">
       <xsd:complexType>
@@ -1062,6 +1062,10 @@
                 <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -1085,6 +1089,28 @@
     <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Balises d’images" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="f66d3a2c-c757-4cdc-87f4-b3c266ce19d8" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="14" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="15" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
@@ -1187,16 +1213,17 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F0FB338B-ED0A-4F1D-9C17-408B90846938}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="911fa86e-1244-486f-9d05-850c48c46759">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{16A7D708-177D-45A8-9A9F-54519F149F23}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -1204,8 +1231,8 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DB4FDE94-F1D1-4D92-9E5B-BE9D0325F69C}">
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5C5B8FBC-63AA-4CAD-8378-E910A0793416}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
@@ -1220,4 +1247,20 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F0FB338B-ED0A-4F1D-9C17-408B90846938}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="911fa86e-1244-486f-9d05-850c48c46759"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Refactor sensitivity payload and supplier risk panels for improved clarity and accuracy
- Updated multiplier_label function to return percentage format for values, enhancing readability.
- Revised supplier risk summary asset descriptions to clarify the impact of supplier sensitivity on product availability.
- Added calculations for input replanning rates and total replanning rates in the global diagnostic payload.
- Enhanced HTML template for better presentation of data, including new styles for secondary tabs and improved hover templates for percentage values.
- Adjusted various labels and descriptions throughout the code to ensure consistency and clarity regarding product availability and service levels.
</commit_message>
<xml_diff>
--- a/etudecas/data/source/268967.xlsx
+++ b/etudecas/data/source/268967.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://scalian-my.sharepoint.com/personal/yannick_martz_scalian_com/Documents/0_FILES_YM/2026/Pierre Fabre/Data/safe/IN/PF/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\lca-simu\etudecas\data\source\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{F1B106E4-76CD-4A29-A43F-305A6627139B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6281DBA4-2371-4798-8153-31371BEB4561}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04810BB8-7A96-4073-BB9F-2465470A5E4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM" sheetId="1" r:id="rId1"/>
@@ -951,7 +951,7 @@
         <v>28</v>
       </c>
       <c r="G6">
-        <v>5000000</v>
+        <v>5000</v>
       </c>
       <c r="H6" t="s">
         <v>29</v>
@@ -1041,15 +1041,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002D5C0BAE13F791428A2467AD4E2CA4A9" ma:contentTypeVersion="8" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="2ef8d77b566c9fd80e9c2bdc9338d629">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="911fa86e-1244-486f-9d05-850c48c46759" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="803aa259af1a7fc7d7bef2888f2078ba" ns2:_="">
     <xsd:import namespace="911fa86e-1244-486f-9d05-850c48c46759"/>
@@ -1213,6 +1204,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1224,14 +1224,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{16A7D708-177D-45A8-9A9F-54519F149F23}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5C5B8FBC-63AA-4CAD-8378-E910A0793416}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1245,6 +1237,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{16A7D708-177D-45A8-9A9F-54519F149F23}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>